<commit_message>
Actualiza el registro y la guía con diez pruebas
Documenta las alertas reutilizables y la suite simplificada. Renueva los diez resultados reales, su cobertura y la planilla académica del equipo Vicente, Victoria y Diego.
</commit_message>
<xml_diff>
--- a/docs/Registro_Pruebas_Unitarias.xlsx
+++ b/docs/Registro_Pruebas_Unitarias.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" r:id="R7ae11486ffef4f70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos de Prueba" sheetId="2" r:id="R8863d31d44804715"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="3" r:id="R8d7536a0093349cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" r:id="Rc7da2d5bc8f64cb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos de Prueba" sheetId="2" r:id="R34549a4d57974547"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="3" r:id="Ra0c253c08ff14a84"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -738,7 +738,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CasosUnitarios" displayName="CasosUnitarios" ref="A1:L48" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CasosUnitarios" displayName="CasosUnitarios" ref="A1:L11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Módulo / Clase"/>
@@ -1163,22 +1163,22 @@
         <x:v>PU-001</x:v>
       </x:c>
       <x:c r="B2" s="44" t="str">
-        <x:v>Almacenamiento</x:v>
+        <x:v>Alerta</x:v>
       </x:c>
       <x:c r="C2" s="44" t="str">
-        <x:v>leerArreglo</x:v>
+        <x:v>Contenido y tipo</x:v>
       </x:c>
       <x:c r="D2" s="44" t="str">
-        <x:v>Error</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="E2" s="44" t="str">
-        <x:v>Recupera almacenamiento inválido</x:v>
+        <x:v>Alerta muestra un mensaje de éxito</x:v>
       </x:c>
       <x:c r="F2" s="44" t="str">
-        <x:v>JSON corrupto y objeto en una clave de arreglo</x:v>
+        <x:v>Texto Guardado y tipo success</x:v>
       </x:c>
       <x:c r="G2" s="44" t="str">
-        <x:v>Devuelve [] sin lanzar errores</x:v>
+        <x:v>Texto, color success y role status</x:v>
       </x:c>
       <x:c r="H2" s="44" t="str">
         <x:v>Todas las aserciones del caso se aprobaron</x:v>
@@ -1193,7 +1193,7 @@
         <x:v>2026-10-14T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="L2" s="44" t="str">
-        <x:v>Duración: 6 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
+        <x:v>Duración: 38 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="78.75" hidden="0" customHeight="1">
@@ -1201,22 +1201,22 @@
         <x:v>PU-002</x:v>
       </x:c>
       <x:c r="B3" s="44" t="str">
-        <x:v>Carrito</x:v>
+        <x:v>Alerta</x:v>
       </x:c>
       <x:c r="C3" s="44" t="str">
-        <x:v>normalizarCarrito</x:v>
+        <x:v>Visibilidad</x:v>
       </x:c>
       <x:c r="D3" s="44" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Borde</x:v>
       </x:c>
       <x:c r="E3" s="44" t="str">
-        <x:v>Normaliza carrito con el catálogo vigente</x:v>
+        <x:v>Alerta permite ocultar y mostrar el contenido</x:v>
       </x:c>
       <x:c r="F3" s="44" t="str">
-        <x:v>Cantidad 2, precio alterado y producto inexistente</x:v>
+        <x:v>visible false y luego true</x:v>
       </x:c>
       <x:c r="G3" s="44" t="str">
-        <x:v>Conserva el producto disponible, cantidad 2 y precio de catálogo</x:v>
+        <x:v>Oculta al inicio y visible después</x:v>
       </x:c>
       <x:c r="H3" s="44" t="str">
         <x:v>Todas las aserciones del caso se aprobaron</x:v>
@@ -1231,7 +1231,7 @@
         <x:v>2026-10-14T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="L3" s="44" t="str">
-        <x:v>Duración: 2 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
+        <x:v>Duración: 7 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="78.75" hidden="0" customHeight="1">
@@ -1239,22 +1239,22 @@
         <x:v>PU-003</x:v>
       </x:c>
       <x:c r="B4" s="44" t="str">
-        <x:v>Carrito</x:v>
+        <x:v>AlertaFormulario</x:v>
       </x:c>
       <x:c r="C4" s="44" t="str">
-        <x:v>agregarAlCarrito</x:v>
+        <x:v>Mensaje vacío</x:v>
       </x:c>
       <x:c r="D4" s="44" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Borde</x:v>
       </x:c>
       <x:c r="E4" s="44" t="str">
-        <x:v>Acumula productos sin mutar el carrito anterior</x:v>
+        <x:v>AlertaFormulario se oculta sin mensaje</x:v>
       </x:c>
       <x:c r="F4" s="44" t="str">
-        <x:v>Una unidad existente y tres añadidas</x:v>
+        <x:v>mensaje null</x:v>
       </x:c>
       <x:c r="G4" s="44" t="str">
-        <x:v>Una fila con cuatro unidades; entrada original intacta</x:v>
+        <x:v>Alerta vacía y oculta</x:v>
       </x:c>
       <x:c r="H4" s="44" t="str">
         <x:v>Todas las aserciones del caso se aprobaron</x:v>
@@ -1269,7 +1269,7 @@
         <x:v>2026-10-14T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="L4" s="44" t="str">
-        <x:v>Duración: 1 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
+        <x:v>Duración: 4 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="78.75" hidden="0" customHeight="1">
@@ -1277,22 +1277,22 @@
         <x:v>PU-004</x:v>
       </x:c>
       <x:c r="B5" s="44" t="str">
-        <x:v>Carrito</x:v>
+        <x:v>AlertaFormulario</x:v>
       </x:c>
       <x:c r="C5" s="44" t="str">
-        <x:v>agregarAlCarrito</x:v>
+        <x:v>Errores y referencia React</x:v>
       </x:c>
       <x:c r="D5" s="44" t="str">
         <x:v>Error</x:v>
       </x:c>
       <x:c r="E5" s="44" t="str">
-        <x:v>Rechaza cantidades inválidas</x:v>
+        <x:v>AlertaFormulario muestra varios errores</x:v>
       </x:c>
       <x:c r="F5" s="44" t="str">
-        <x:v>Cero, fracción y NaN</x:v>
+        <x:v>Dos errores y una referencia React</x:v>
       </x:c>
       <x:c r="G5" s="44" t="str">
-        <x:v>Lanza error y no agrega productos</x:v>
+        <x:v>Dos textos separados por br, role alert y ref al elemento</x:v>
       </x:c>
       <x:c r="H5" s="44" t="str">
         <x:v>Todas las aserciones del caso se aprobaron</x:v>
@@ -1307,7 +1307,7 @@
         <x:v>2026-10-14T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="L5" s="44" t="str">
-        <x:v>Duración: 1 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
+        <x:v>Duración: 10 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="78.75" hidden="0" customHeight="1">
@@ -1315,22 +1315,22 @@
         <x:v>PU-005</x:v>
       </x:c>
       <x:c r="B6" s="44" t="str">
-        <x:v>Carrito</x:v>
+        <x:v>Notificacion</x:v>
       </x:c>
       <x:c r="C6" s="44" t="str">
-        <x:v>cambiarCantidadCarrito</x:v>
+        <x:v>Contenido recibido</x:v>
       </x:c>
       <x:c r="D6" s="44" t="str">
-        <x:v>Borde</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="E6" s="44" t="str">
-        <x:v>Quita el producto al disminuir su última unidad</x:v>
+        <x:v>Notificacion recibe su contenido</x:v>
       </x:c>
       <x:c r="F6" s="44" t="str">
-        <x:v>Carrito con una unidad; variación -1</x:v>
+        <x:v>Texto Producto agregado</x:v>
       </x:c>
       <x:c r="G6" s="44" t="str">
-        <x:v>Carrito vacío</x:v>
+        <x:v>Texto recibido y role status</x:v>
       </x:c>
       <x:c r="H6" s="44" t="str">
         <x:v>Todas las aserciones del caso se aprobaron</x:v>
@@ -1345,7 +1345,7 @@
         <x:v>2026-10-14T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="L6" s="44" t="str">
-        <x:v>Duración: 1 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
+        <x:v>Duración: 4 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="78.75" hidden="0" customHeight="1">
@@ -1353,22 +1353,22 @@
         <x:v>PU-006</x:v>
       </x:c>
       <x:c r="B7" s="44" t="str">
-        <x:v>Precios</x:v>
+        <x:v>TarjetasProductos</x:v>
       </x:c>
       <x:c r="C7" s="44" t="str">
-        <x:v>precioFinal / totalCarrito</x:v>
+        <x:v>Producto y descuento</x:v>
       </x:c>
       <x:c r="D7" s="44" t="str">
-        <x:v>Borde</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="E7" s="44" t="str">
-        <x:v>Calcula descuentos y totales en pesos enteros</x:v>
+        <x:v>Tarjetas muestra el producto y su descuento</x:v>
       </x:c>
       <x:c r="F7" s="44" t="str">
-        <x:v>Precio 10000, descuento 20%, cantidad 2; descuento 100%</x:v>
+        <x:v>Producto de 10000 con descuento 20%</x:v>
       </x:c>
       <x:c r="G7" s="44" t="str">
-        <x:v>Precio 8000, total 16000 y precio cero al 100%</x:v>
+        <x:v>Nombre y precio final 8000</x:v>
       </x:c>
       <x:c r="H7" s="44" t="str">
         <x:v>Todas las aserciones del caso se aprobaron</x:v>
@@ -1383,7 +1383,7 @@
         <x:v>2026-10-14T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="L7" s="44" t="str">
-        <x:v>Duración: 1 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
+        <x:v>Duración: 61 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="78.75" hidden="0" customHeight="1">
@@ -1391,22 +1391,22 @@
         <x:v>PU-007</x:v>
       </x:c>
       <x:c r="B8" s="44" t="str">
-        <x:v>Productos</x:v>
+        <x:v>TarjetasProductos</x:v>
       </x:c>
       <x:c r="C8" s="44" t="str">
-        <x:v>crear / editar / eliminarProducto</x:v>
+        <x:v>Evento agregar / callback</x:v>
       </x:c>
       <x:c r="D8" s="44" t="str">
         <x:v>Normal</x:v>
       </x:c>
       <x:c r="E8" s="44" t="str">
-        <x:v>Completa CRUD sin cambiar el identificador al editar</x:v>
+        <x:v>Agregar al carrito llama a la notificación</x:v>
       </x:c>
       <x:c r="F8" s="44" t="str">
-        <x:v>Crear, editar categoría a salados y eliminar</x:v>
+        <x:v>Clic Agregar al carrito y callback spy</x:v>
       </x:c>
       <x:c r="G8" s="44" t="str">
-        <x:v>Persistencia actualizada; ID estable; producto eliminado</x:v>
+        <x:v>Una llamada y producto guardado</x:v>
       </x:c>
       <x:c r="H8" s="44" t="str">
         <x:v>Todas las aserciones del caso se aprobaron</x:v>
@@ -1421,7 +1421,7 @@
         <x:v>2026-10-14T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="L8" s="44" t="str">
-        <x:v>Duración: 2 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
+        <x:v>Duración: 10 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="78.75" hidden="0" customHeight="1">
@@ -1429,22 +1429,22 @@
         <x:v>PU-008</x:v>
       </x:c>
       <x:c r="B9" s="44" t="str">
-        <x:v>Productos</x:v>
+        <x:v>CatalogoProductos</x:v>
       </x:c>
       <x:c r="C9" s="44" t="str">
-        <x:v>crear / editar / eliminarProducto</x:v>
+        <x:v>Evento búsqueda</x:v>
       </x:c>
       <x:c r="D9" s="44" t="str">
-        <x:v>Error</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="E9" s="44" t="str">
-        <x:v>Valida datos e identificadores en administración</x:v>
+        <x:v>La búsqueda filtra el catálogo</x:v>
       </x:c>
       <x:c r="F9" s="44" t="str">
-        <x:v>Precio negativo, descuento 101 e ID desconocido</x:v>
+        <x:v>Escribir FRUTILLA</x:v>
       </x:c>
       <x:c r="G9" s="44" t="str">
-        <x:v>Errores sin sobrescribir datos</x:v>
+        <x:v>Una tarjeta de Pastel de Frutilla</x:v>
       </x:c>
       <x:c r="H9" s="44" t="str">
         <x:v>Todas las aserciones del caso se aprobaron</x:v>
@@ -1459,7 +1459,7 @@
         <x:v>2026-10-14T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="L9" s="44" t="str">
-        <x:v>Duración: 1 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
+        <x:v>Duración: 70 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="78.75" hidden="0" customHeight="1">
@@ -1467,22 +1467,22 @@
         <x:v>PU-009</x:v>
       </x:c>
       <x:c r="B10" s="44" t="str">
-        <x:v>Autenticación</x:v>
+        <x:v>FilasCarrito</x:v>
       </x:c>
       <x:c r="C10" s="44" t="str">
-        <x:v>registrarUsuario</x:v>
+        <x:v>Carrito vacío</x:v>
       </x:c>
       <x:c r="D10" s="44" t="str">
-        <x:v>Error</x:v>
+        <x:v>Borde</x:v>
       </x:c>
       <x:c r="E10" s="44" t="str">
-        <x:v>Valida un registro vacío</x:v>
+        <x:v>El carrito vacío muestra una alerta</x:v>
       </x:c>
       <x:c r="F10" s="44" t="str">
-        <x:v>Formulario sin campos</x:v>
+        <x:v>Carrito sin productos</x:v>
       </x:c>
       <x:c r="G10" s="44" t="str">
-        <x:v>Lista de errores; no crea usuario</x:v>
+        <x:v>Mensaje informativo de carrito vacío</x:v>
       </x:c>
       <x:c r="H10" s="44" t="str">
         <x:v>Todas las aserciones del caso se aprobaron</x:v>
@@ -1497,7 +1497,7 @@
         <x:v>2026-10-14T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="L10" s="44" t="str">
-        <x:v>Duración: 1 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
+        <x:v>Duración: 2 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="78.75" hidden="0" customHeight="1">
@@ -1505,22 +1505,22 @@
         <x:v>PU-010</x:v>
       </x:c>
       <x:c r="B11" s="44" t="str">
-        <x:v>Autenticación</x:v>
+        <x:v>FormularioProducto</x:v>
       </x:c>
       <x:c r="C11" s="44" t="str">
-        <x:v>registrarUsuario</x:v>
+        <x:v>Props y evento submit</x:v>
       </x:c>
       <x:c r="D11" s="44" t="str">
-        <x:v>Borde</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="E11" s="44" t="str">
-        <x:v>Normaliza correo y evita registros duplicados</x:v>
+        <x:v>FormularioProducto entrega el precio editado</x:v>
       </x:c>
       <x:c r="F11" s="44" t="str">
-        <x:v>Correo ANA@example.test y rol admin enviado por el cliente</x:v>
+        <x:v>Producto recibido por props y precio 15000</x:v>
       </x:c>
       <x:c r="G11" s="44" t="str">
-        <x:v>Correo en minúsculas, rol cliente y segundo registro rechazado</x:v>
+        <x:v>Nombre precargado y callback con precio 15000</x:v>
       </x:c>
       <x:c r="H11" s="44" t="str">
         <x:v>Todas las aserciones del caso se aprobaron</x:v>
@@ -1535,1414 +1535,526 @@
         <x:v>2026-10-14T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="L11" s="44" t="str">
-        <x:v>Duración: 2 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A12" s="44" t="str">
-        <x:v>PU-011</x:v>
-      </x:c>
-      <x:c r="B12" s="44" t="str">
-        <x:v>Autenticación</x:v>
-      </x:c>
-      <x:c r="C12" s="44" t="str">
-        <x:v>iniciarSesion</x:v>
-      </x:c>
-      <x:c r="D12" s="44" t="str">
-        <x:v>Error</x:v>
-      </x:c>
-      <x:c r="E12" s="44" t="str">
-        <x:v>Rechaza credenciales incorrectas</x:v>
-      </x:c>
-      <x:c r="F12" s="44" t="str">
-        <x:v>Usuario registrado y contraseña incorrecta</x:v>
-      </x:c>
-      <x:c r="G12" s="44" t="str">
-        <x:v>Error; sesión inexistente; solicita limpiar contraseña</x:v>
-      </x:c>
-      <x:c r="H12" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I12" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J12" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K12" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L12" s="44" t="str">
-        <x:v>Duración: 1 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A13" s="44" t="str">
-        <x:v>PU-012</x:v>
-      </x:c>
-      <x:c r="B13" s="44" t="str">
-        <x:v>Autenticación</x:v>
-      </x:c>
-      <x:c r="C13" s="44" t="str">
-        <x:v>iniciarSesion</x:v>
-      </x:c>
-      <x:c r="D13" s="44" t="str">
-        <x:v>Normal</x:v>
-      </x:c>
-      <x:c r="E13" s="44" t="str">
-        <x:v>Guarda sesión temporal sin contraseña</x:v>
-      </x:c>
-      <x:c r="F13" s="44" t="str">
-        <x:v>Login válido sin recordar cuenta</x:v>
-      </x:c>
-      <x:c r="G13" s="44" t="str">
-        <x:v>sessionStorage contiene usuario; localStorage no; sin password</x:v>
-      </x:c>
-      <x:c r="H13" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I13" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J13" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K13" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L13" s="44" t="str">
-        <x:v>Duración: 1 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A14" s="44" t="str">
-        <x:v>PU-013</x:v>
-      </x:c>
-      <x:c r="B14" s="44" t="str">
-        <x:v>Autenticación</x:v>
-      </x:c>
-      <x:c r="C14" s="44" t="str">
-        <x:v>iniciarSesion / obtenerUsuarioActivo</x:v>
-      </x:c>
-      <x:c r="D14" s="44" t="str">
-        <x:v>Error</x:v>
-      </x:c>
-      <x:c r="E14" s="44" t="str">
-        <x:v>Guarda la cuenta recordada y recupera sesión corrupta</x:v>
-      </x:c>
-      <x:c r="F14" s="44" t="str">
-        <x:v>Login con recordarCuenta; luego JSON corrupto</x:v>
-      </x:c>
-      <x:c r="G14" s="44" t="str">
-        <x:v>Sesión en localStorage; dato inválido se limpia</x:v>
-      </x:c>
-      <x:c r="H14" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I14" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J14" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K14" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L14" s="44" t="str">
-        <x:v>Duración: 0 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A15" s="44" t="str">
-        <x:v>PU-014</x:v>
-      </x:c>
-      <x:c r="B15" s="44" t="str">
-        <x:v>Autenticación</x:v>
-      </x:c>
-      <x:c r="C15" s="44" t="str">
-        <x:v>crearAdministradorDemo</x:v>
-      </x:c>
-      <x:c r="D15" s="44" t="str">
-        <x:v>Borde</x:v>
-      </x:c>
-      <x:c r="E15" s="44" t="str">
-        <x:v>Crea administrador demo sin duplicados</x:v>
-      </x:c>
-      <x:c r="F15" s="44" t="str">
-        <x:v>Dos inicializaciones del administrador</x:v>
-      </x:c>
-      <x:c r="G15" s="44" t="str">
-        <x:v>Una sola cuenta con rol admin</x:v>
-      </x:c>
-      <x:c r="H15" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I15" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J15" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K15" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L15" s="44" t="str">
-        <x:v>Duración: 1 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A16" s="44" t="str">
-        <x:v>PU-015</x:v>
-      </x:c>
-      <x:c r="B16" s="44" t="str">
-        <x:v>Consultas</x:v>
-      </x:c>
-      <x:c r="C16" s="44" t="str">
-        <x:v>registrarConsulta / cambiarEstadoConsulta</x:v>
-      </x:c>
-      <x:c r="D16" s="44" t="str">
-        <x:v>Normal</x:v>
-      </x:c>
-      <x:c r="E16" s="44" t="str">
-        <x:v>Normaliza consultas y actualiza su estado</x:v>
-      </x:c>
-      <x:c r="F16" s="44" t="str">
-        <x:v>Correo en mayúsculas y consulta con espacios</x:v>
-      </x:c>
-      <x:c r="G16" s="44" t="str">
-        <x:v>Datos recortados, estado pendiente y posterior resuelta</x:v>
-      </x:c>
-      <x:c r="H16" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I16" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J16" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K16" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L16" s="44" t="str">
-        <x:v>Duración: 5 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A17" s="44" t="str">
-        <x:v>PU-016</x:v>
-      </x:c>
-      <x:c r="B17" s="44" t="str">
-        <x:v>Consultas</x:v>
-      </x:c>
-      <x:c r="C17" s="44" t="str">
-        <x:v>registrarConsulta</x:v>
-      </x:c>
-      <x:c r="D17" s="44" t="str">
-        <x:v>Error</x:v>
-      </x:c>
-      <x:c r="E17" s="44" t="str">
-        <x:v>No guarda consultas vacías</x:v>
-      </x:c>
-      <x:c r="F17" s="44" t="str">
-        <x:v>Mensaje compuesto por espacios</x:v>
-      </x:c>
-      <x:c r="G17" s="44" t="str">
-        <x:v>Advertencia y almacenamiento sin consultas</x:v>
-      </x:c>
-      <x:c r="H17" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I17" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J17" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K17" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L17" s="44" t="str">
-        <x:v>Duración: 1 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A18" s="44" t="str">
-        <x:v>PU-017</x:v>
-      </x:c>
-      <x:c r="B18" s="44" t="str">
-        <x:v>Pedidos</x:v>
-      </x:c>
-      <x:c r="C18" s="44" t="str">
-        <x:v>crearPedido</x:v>
-      </x:c>
-      <x:c r="D18" s="44" t="str">
-        <x:v>Normal</x:v>
-      </x:c>
-      <x:c r="E18" s="44" t="str">
-        <x:v>Registra total, entrega y precios pagados</x:v>
-      </x:c>
-      <x:c r="F18" s="44" t="str">
-        <x:v>Dos unidades de 10000 con 20% de descuento y despacho de 3000</x:v>
-      </x:c>
-      <x:c r="G18" s="44" t="str">
-        <x:v>Subtotal 16000; total 19000; snapshot de precio final 8000</x:v>
-      </x:c>
-      <x:c r="H18" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I18" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J18" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K18" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L18" s="44" t="str">
-        <x:v>Duración: 2 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A19" s="44" t="str">
-        <x:v>PU-018</x:v>
-      </x:c>
-      <x:c r="B19" s="44" t="str">
-        <x:v>Pedidos</x:v>
-      </x:c>
-      <x:c r="C19" s="44" t="str">
-        <x:v>crearPedido</x:v>
-      </x:c>
-      <x:c r="D19" s="44" t="str">
-        <x:v>Error</x:v>
-      </x:c>
-      <x:c r="E19" s="44" t="str">
-        <x:v>Pago rechazado no crea pedido</x:v>
-      </x:c>
-      <x:c r="F19" s="44" t="str">
-        <x:v>Carrito válido y pago rechazado</x:v>
-      </x:c>
-      <x:c r="G19" s="44" t="str">
-        <x:v>Resultado aprobado false; pedidos sin cambios</x:v>
-      </x:c>
-      <x:c r="H19" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I19" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J19" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K19" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L19" s="44" t="str">
-        <x:v>Duración: 1 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A20" s="44" t="str">
-        <x:v>PU-019</x:v>
-      </x:c>
-      <x:c r="B20" s="44" t="str">
-        <x:v>Pedidos</x:v>
-      </x:c>
-      <x:c r="C20" s="44" t="str">
-        <x:v>crearPedido</x:v>
-      </x:c>
-      <x:c r="D20" s="44" t="str">
-        <x:v>Error</x:v>
-      </x:c>
-      <x:c r="E20" s="44" t="str">
-        <x:v>Rechaza compras vacías o con datos inválidos</x:v>
-      </x:c>
-      <x:c r="F20" s="44" t="str">
-        <x:v>Carrito vacío, email inválido y producto eliminado</x:v>
-      </x:c>
-      <x:c r="G20" s="44" t="str">
-        <x:v>Lanza errores; no persiste pedidos</x:v>
-      </x:c>
-      <x:c r="H20" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I20" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J20" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K20" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L20" s="44" t="str">
-        <x:v>Duración: 2 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A21" s="44" t="str">
-        <x:v>PU-020</x:v>
-      </x:c>
-      <x:c r="B21" s="44" t="str">
-        <x:v>Pedidos</x:v>
-      </x:c>
-      <x:c r="C21" s="44" t="str">
-        <x:v>pedidosDelUsuario</x:v>
-      </x:c>
-      <x:c r="D21" s="44" t="str">
-        <x:v>Normal</x:v>
-      </x:c>
-      <x:c r="E21" s="44" t="str">
-        <x:v>Historial muestra pedidos del usuario correspondiente</x:v>
-      </x:c>
-      <x:c r="F21" s="44" t="str">
-        <x:v>Pedidos de Ana y de otra persona</x:v>
-      </x:c>
-      <x:c r="G21" s="44" t="str">
-        <x:v>Cada historial contiene solamente su pedido</x:v>
-      </x:c>
-      <x:c r="H21" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I21" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J21" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K21" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L21" s="44" t="str">
-        <x:v>Duración: 2 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A22" s="44" t="str">
-        <x:v>PU-021</x:v>
-      </x:c>
-      <x:c r="B22" s="44" t="str">
-        <x:v>TarjetasProductos</x:v>
-      </x:c>
-      <x:c r="C22" s="44" t="str">
-        <x:v>Renderizado</x:v>
-      </x:c>
-      <x:c r="D22" s="44" t="str">
-        <x:v>Normal</x:v>
-      </x:c>
-      <x:c r="E22" s="44" t="str">
-        <x:v>Tarjetas renderiza los datos recibidos por props</x:v>
-      </x:c>
-      <x:c r="F22" s="44" t="str">
-        <x:v>Producto Pastel de prueba, precio 10000 y descuento 20%</x:v>
-      </x:c>
-      <x:c r="G22" s="44" t="str">
-        <x:v>Nombre y precio final 8000 en una tarjeta</x:v>
-      </x:c>
-      <x:c r="H22" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I22" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J22" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K22" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L22" s="44" t="str">
-        <x:v>Duración: 76 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A23" s="44" t="str">
-        <x:v>PU-022</x:v>
-      </x:c>
-      <x:c r="B23" s="44" t="str">
-        <x:v>TarjetasProductos</x:v>
-      </x:c>
-      <x:c r="C23" s="44" t="str">
-        <x:v>Evento agregar / callback</x:v>
-      </x:c>
-      <x:c r="D23" s="44" t="str">
-        <x:v>Normal</x:v>
-      </x:c>
-      <x:c r="E23" s="44" t="str">
-        <x:v>Evento agregar ejecuta callback y actualiza el carrito</x:v>
-      </x:c>
-      <x:c r="F23" s="44" t="str">
-        <x:v>Clic en Agregar al carrito; callback spy</x:v>
-      </x:c>
-      <x:c r="G23" s="44" t="str">
-        <x:v>Notifica una vez y persiste el producto correcto</x:v>
-      </x:c>
-      <x:c r="H23" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I23" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J23" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K23" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L23" s="44" t="str">
-        <x:v>Duración: 9 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A24" s="44" t="str">
-        <x:v>PU-023</x:v>
-      </x:c>
-      <x:c r="B24" s="44" t="str">
-        <x:v>Notificacion</x:v>
-      </x:c>
-      <x:c r="C24" s="44" t="str">
-        <x:v>Renderizado de props</x:v>
-      </x:c>
-      <x:c r="D24" s="44" t="str">
-        <x:v>Normal</x:v>
-      </x:c>
-      <x:c r="E24" s="44" t="str">
-        <x:v>Notificación usa contenido y atributos recibidos</x:v>
-      </x:c>
-      <x:c r="F24" s="44" t="str">
-        <x:v>Children Consulta enviada, ID aviso y role status</x:v>
-      </x:c>
-      <x:c r="G24" s="44" t="str">
-        <x:v>Contenido y atributos presentes en el DOM</x:v>
-      </x:c>
-      <x:c r="H24" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I24" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J24" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K24" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L24" s="44" t="str">
-        <x:v>Duración: 2 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A25" s="44" t="str">
-        <x:v>PU-024</x:v>
-      </x:c>
-      <x:c r="B25" s="44" t="str">
-        <x:v>CatalogoProductos</x:v>
-      </x:c>
-      <x:c r="C25" s="44" t="str">
-        <x:v>Filtro de categoría</x:v>
-      </x:c>
-      <x:c r="D25" s="44" t="str">
-        <x:v>Normal</x:v>
-      </x:c>
-      <x:c r="E25" s="44" t="str">
-        <x:v>Catálogo renderiza solamente su categoría</x:v>
-      </x:c>
-      <x:c r="F25" s="44" t="str">
-        <x:v>Categoría pasteleria y catálogo inicial de doce productos</x:v>
-      </x:c>
-      <x:c r="G25" s="44" t="str">
-        <x:v>Tres tarjetas de pastelería</x:v>
-      </x:c>
-      <x:c r="H25" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I25" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J25" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K25" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L25" s="44" t="str">
-        <x:v>Duración: 66 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A26" s="44" t="str">
-        <x:v>PU-025</x:v>
-      </x:c>
-      <x:c r="B26" s="44" t="str">
-        <x:v>CatalogoProductos</x:v>
-      </x:c>
-      <x:c r="C26" s="44" t="str">
-        <x:v>Evento búsqueda</x:v>
-      </x:c>
-      <x:c r="D26" s="44" t="str">
-        <x:v>Normal</x:v>
-      </x:c>
-      <x:c r="E26" s="44" t="str">
-        <x:v>Búsqueda reacciona al estado del input</x:v>
-      </x:c>
-      <x:c r="F26" s="44" t="str">
-        <x:v>Escribir FRUTILLA</x:v>
-      </x:c>
-      <x:c r="G26" s="44" t="str">
-        <x:v>Una tarjeta de Pastel de Frutilla</x:v>
-      </x:c>
-      <x:c r="H26" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I26" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J26" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K26" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L26" s="44" t="str">
-        <x:v>Duración: 20 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A27" s="44" t="str">
-        <x:v>PU-026</x:v>
-      </x:c>
-      <x:c r="B27" s="44" t="str">
-        <x:v>CatalogoProductos</x:v>
-      </x:c>
-      <x:c r="C27" s="44" t="str">
-        <x:v>Estado sin resultados</x:v>
-      </x:c>
-      <x:c r="D27" s="44" t="str">
-        <x:v>Borde</x:v>
-      </x:c>
-      <x:c r="E27" s="44" t="str">
-        <x:v>Catálogo muestra el estado sin resultados</x:v>
-      </x:c>
-      <x:c r="F27" s="44" t="str">
-        <x:v>Buscar un producto inexistente</x:v>
-      </x:c>
-      <x:c r="G27" s="44" t="str">
-        <x:v>Mensaje visible y cero tarjetas</x:v>
-      </x:c>
-      <x:c r="H27" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I27" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J27" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K27" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L27" s="44" t="str">
-        <x:v>Duración: 15 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A28" s="44" t="str">
-        <x:v>PU-027</x:v>
-      </x:c>
-      <x:c r="B28" s="44" t="str">
-        <x:v>CatalogoProductos</x:v>
-      </x:c>
-      <x:c r="C28" s="44" t="str">
-        <x:v>Evento orden</x:v>
-      </x:c>
-      <x:c r="D28" s="44" t="str">
-        <x:v>Normal</x:v>
-      </x:c>
-      <x:c r="E28" s="44" t="str">
-        <x:v>Orden del catálogo responde al select</x:v>
-      </x:c>
-      <x:c r="F28" s="44" t="str">
-        <x:v>Seleccionar menor precio</x:v>
-      </x:c>
-      <x:c r="G28" s="44" t="str">
-        <x:v>Pastel de Vainilla en primer lugar</x:v>
-      </x:c>
-      <x:c r="H28" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I28" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J28" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K28" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L28" s="44" t="str">
-        <x:v>Duración: 12 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A29" s="44" t="str">
-        <x:v>PU-028</x:v>
-      </x:c>
-      <x:c r="B29" s="44" t="str">
-        <x:v>Carrito</x:v>
-      </x:c>
-      <x:c r="C29" s="44" t="str">
-        <x:v>Renderizado vacío</x:v>
-      </x:c>
-      <x:c r="D29" s="44" t="str">
-        <x:v>Borde</x:v>
-      </x:c>
-      <x:c r="E29" s="44" t="str">
-        <x:v>Carrito vacío oculta acciones de compra</x:v>
-      </x:c>
-      <x:c r="F29" s="44" t="str">
-        <x:v>Sin productos guardados</x:v>
-      </x:c>
-      <x:c r="G29" s="44" t="str">
-        <x:v>Mensaje de carrito vacío y sin botón Vaciar carrito</x:v>
-      </x:c>
-      <x:c r="H29" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I29" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J29" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K29" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L29" s="44" t="str">
         <x:v>Duración: 7 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A30" s="44" t="str">
-        <x:v>PU-029</x:v>
-      </x:c>
-      <x:c r="B30" s="44" t="str">
-        <x:v>Carrito</x:v>
-      </x:c>
-      <x:c r="C30" s="44" t="str">
-        <x:v>Evento disminuir</x:v>
-      </x:c>
-      <x:c r="D30" s="44" t="str">
-        <x:v>Borde</x:v>
-      </x:c>
-      <x:c r="E30" s="44" t="str">
-        <x:v>Carrito actualiza cantidades y elimina la última unidad</x:v>
-      </x:c>
-      <x:c r="F30" s="44" t="str">
-        <x:v>Dos unidades con precio final 8000; dos clics en disminuir</x:v>
-      </x:c>
-      <x:c r="G30" s="44" t="str">
-        <x:v>Totales 16000, 8000 y cero; carrito vacío</x:v>
-      </x:c>
-      <x:c r="H30" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I30" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J30" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K30" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L30" s="44" t="str">
-        <x:v>Duración: 15 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A31" s="44" t="str">
-        <x:v>PU-030</x:v>
-      </x:c>
-      <x:c r="B31" s="44" t="str">
-        <x:v>DetalleProducto</x:v>
-      </x:c>
-      <x:c r="C31" s="44" t="str">
-        <x:v>Producto inexistente</x:v>
-      </x:c>
-      <x:c r="D31" s="44" t="str">
-        <x:v>Error</x:v>
-      </x:c>
-      <x:c r="E31" s="44" t="str">
-        <x:v>Detalle resuelve identificadores inexistentes</x:v>
-      </x:c>
-      <x:c r="F31" s="44" t="str">
-        <x:v>URL /producto/no-existe</x:v>
-      </x:c>
-      <x:c r="G31" s="44" t="str">
-        <x:v>Mensaje de producto no disponible</x:v>
-      </x:c>
-      <x:c r="H31" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I31" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J31" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K31" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L31" s="44" t="str">
-        <x:v>Duración: 13 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A32" s="44" t="str">
-        <x:v>PU-031</x:v>
-      </x:c>
-      <x:c r="B32" s="44" t="str">
-        <x:v>DetalleProducto</x:v>
-      </x:c>
-      <x:c r="C32" s="44" t="str">
-        <x:v>Parámetro y evento agregar</x:v>
-      </x:c>
-      <x:c r="D32" s="44" t="str">
-        <x:v>Normal</x:v>
-      </x:c>
-      <x:c r="E32" s="44" t="str">
-        <x:v>Detalle usa el parámetro y añade la cantidad elegida</x:v>
-      </x:c>
-      <x:c r="F32" s="44" t="str">
-        <x:v>Producto existente, cantidad 3 y clic agregar</x:v>
-      </x:c>
-      <x:c r="G32" s="44" t="str">
-        <x:v>Carrito de tres unidades y notificación visible</x:v>
-      </x:c>
-      <x:c r="H32" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I32" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J32" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K32" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L32" s="44" t="str">
-        <x:v>Duración: 52 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A33" s="44" t="str">
-        <x:v>PU-032</x:v>
-      </x:c>
-      <x:c r="B33" s="44" t="str">
-        <x:v>DetalleProducto</x:v>
-      </x:c>
-      <x:c r="C33" s="44" t="str">
-        <x:v>Validación de cantidad</x:v>
-      </x:c>
-      <x:c r="D33" s="44" t="str">
-        <x:v>Error</x:v>
-      </x:c>
-      <x:c r="E33" s="44" t="str">
-        <x:v>Detalle rechaza cantidades fraccionarias</x:v>
-      </x:c>
-      <x:c r="F33" s="44" t="str">
-        <x:v>Cantidad 1.5</x:v>
-      </x:c>
-      <x:c r="G33" s="44" t="str">
-        <x:v>Reinicia a una unidad, enfoca el input y no agrega</x:v>
-      </x:c>
-      <x:c r="H33" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I33" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J33" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K33" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L33" s="44" t="str">
-        <x:v>Duración: 18 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A34" s="44" t="str">
-        <x:v>PU-033</x:v>
-      </x:c>
-      <x:c r="B34" s="44" t="str">
-        <x:v>RegistroUsuario</x:v>
-      </x:c>
-      <x:c r="C34" s="44" t="str">
-        <x:v>Mensajes de validación</x:v>
-      </x:c>
-      <x:c r="D34" s="44" t="str">
-        <x:v>Error</x:v>
-      </x:c>
-      <x:c r="E34" s="44" t="str">
-        <x:v>Registro muestra errores condicionalmente</x:v>
-      </x:c>
-      <x:c r="F34" s="44" t="str">
-        <x:v>Formulario inicialmente vacío y luego submit</x:v>
-      </x:c>
-      <x:c r="G34" s="44" t="str">
-        <x:v>Mensaje oculto al inicio; errores visibles después; sin usuario creado</x:v>
-      </x:c>
-      <x:c r="H34" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I34" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J34" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K34" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L34" s="44" t="str">
-        <x:v>Duración: 34 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A35" s="44" t="str">
-        <x:v>PU-034</x:v>
-      </x:c>
-      <x:c r="B35" s="44" t="str">
-        <x:v>RegistroUsuario</x:v>
-      </x:c>
-      <x:c r="C35" s="44" t="str">
-        <x:v>Evento submit</x:v>
-      </x:c>
-      <x:c r="D35" s="44" t="str">
-        <x:v>Normal</x:v>
-      </x:c>
-      <x:c r="E35" s="44" t="str">
-        <x:v>Registro guarda datos y limpia el formulario</x:v>
-      </x:c>
-      <x:c r="F35" s="44" t="str">
-        <x:v>Campos válidos introducidos con eventos de input</x:v>
-      </x:c>
-      <x:c r="G35" s="44" t="str">
-        <x:v>Cuenta cliente persistida y mensaje de éxito</x:v>
-      </x:c>
-      <x:c r="H35" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I35" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J35" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K35" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L35" s="44" t="str">
-        <x:v>Duración: 26 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A36" s="44" t="str">
-        <x:v>PU-035</x:v>
-      </x:c>
-      <x:c r="B36" s="44" t="str">
-        <x:v>InicioSesion</x:v>
-      </x:c>
-      <x:c r="C36" s="44" t="str">
-        <x:v>Credenciales inválidas</x:v>
-      </x:c>
-      <x:c r="D36" s="44" t="str">
-        <x:v>Error</x:v>
-      </x:c>
-      <x:c r="E36" s="44" t="str">
-        <x:v>Login inválido limpia y enfoca la contraseña</x:v>
-      </x:c>
-      <x:c r="F36" s="44" t="str">
-        <x:v>Correo válido y contraseña incorrecta</x:v>
-      </x:c>
-      <x:c r="G36" s="44" t="str">
-        <x:v>Mensaje de error, contraseña vacía y foco en su input</x:v>
-      </x:c>
-      <x:c r="H36" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I36" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J36" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K36" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L36" s="44" t="str">
-        <x:v>Duración: 20 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A37" s="44" t="str">
-        <x:v>PU-036</x:v>
-      </x:c>
-      <x:c r="B37" s="44" t="str">
-        <x:v>InicioSesion</x:v>
-      </x:c>
-      <x:c r="C37" s="44" t="str">
-        <x:v>Evento submit / menú</x:v>
-      </x:c>
-      <x:c r="D37" s="44" t="str">
-        <x:v>Normal</x:v>
-      </x:c>
-      <x:c r="E37" s="44" t="str">
-        <x:v>Login actualiza el menú de sesión inmediatamente</x:v>
-      </x:c>
-      <x:c r="F37" s="44" t="str">
-        <x:v>Credenciales válidas</x:v>
-      </x:c>
-      <x:c r="G37" s="44" t="str">
-        <x:v>Hola, Ana aparece y la sesión se guarda sin contraseña</x:v>
-      </x:c>
-      <x:c r="H37" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I37" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J37" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K37" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L37" s="44" t="str">
-        <x:v>Duración: 13 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A38" s="44" t="str">
-        <x:v>PU-037</x:v>
-      </x:c>
-      <x:c r="B38" s="44" t="str">
-        <x:v>Contacto</x:v>
-      </x:c>
-      <x:c r="C38" s="44" t="str">
-        <x:v>Evento submit</x:v>
-      </x:c>
-      <x:c r="D38" s="44" t="str">
-        <x:v>Normal</x:v>
-      </x:c>
-      <x:c r="E38" s="44" t="str">
-        <x:v>Contacto valida, guarda y limpia sus campos</x:v>
-      </x:c>
-      <x:c r="F38" s="44" t="str">
-        <x:v>Mensaje con espacios y luego consulta válida</x:v>
-      </x:c>
-      <x:c r="G38" s="44" t="str">
-        <x:v>Advertencia inicial; consulta persistida y formulario vacío al éxito</x:v>
-      </x:c>
-      <x:c r="H38" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I38" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J38" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K38" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L38" s="44" t="str">
-        <x:v>Duración: 17 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A39" s="44" t="str">
-        <x:v>PU-038</x:v>
-      </x:c>
-      <x:c r="B39" s="44" t="str">
-        <x:v>TablaProductos</x:v>
-      </x:c>
-      <x:c r="C39" s="44" t="str">
-        <x:v>Callbacks de props</x:v>
-      </x:c>
-      <x:c r="D39" s="44" t="str">
-        <x:v>Normal</x:v>
-      </x:c>
-      <x:c r="E39" s="44" t="str">
-        <x:v>Tabla de productos ejecuta callbacks recibidos por props</x:v>
-      </x:c>
-      <x:c r="F39" s="44" t="str">
-        <x:v>Clic editar y eliminación confirmada; callbacks spy</x:v>
-      </x:c>
-      <x:c r="G39" s="44" t="str">
-        <x:v>Editar recibe objeto; eliminar recibe ID solamente al confirmar</x:v>
-      </x:c>
-      <x:c r="H39" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I39" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J39" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K39" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L39" s="44" t="str">
-        <x:v>Duración: 10 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A40" s="44" t="str">
-        <x:v>PU-039</x:v>
-      </x:c>
-      <x:c r="B40" s="44" t="str">
-        <x:v>FormularioProducto</x:v>
-      </x:c>
-      <x:c r="C40" s="44" t="str">
-        <x:v>Props y evento submit</x:v>
-      </x:c>
-      <x:c r="D40" s="44" t="str">
-        <x:v>Normal</x:v>
-      </x:c>
-      <x:c r="E40" s="44" t="str">
-        <x:v>Formulario de edición precarga props y entrega cambios</x:v>
-      </x:c>
-      <x:c r="F40" s="44" t="str">
-        <x:v>Producto inicial y precio modificado a 15000</x:v>
-      </x:c>
-      <x:c r="G40" s="44" t="str">
-        <x:v>Callback recibe datos del formulario con nuevo precio</x:v>
-      </x:c>
-      <x:c r="H40" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I40" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J40" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K40" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L40" s="44" t="str">
-        <x:v>Duración: 11 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A41" s="44" t="str">
-        <x:v>PU-040</x:v>
-      </x:c>
-      <x:c r="B41" s="44" t="str">
-        <x:v>App</x:v>
-      </x:c>
-      <x:c r="C41" s="44" t="str">
-        <x:v>Protección de acceso</x:v>
-      </x:c>
-      <x:c r="D41" s="44" t="str">
-        <x:v>Error</x:v>
-      </x:c>
-      <x:c r="E41" s="44" t="str">
-        <x:v>Las rutas protegidas bloquean visitantes y clientes</x:v>
-      </x:c>
-      <x:c r="F41" s="44" t="str">
-        <x:v>Entrar a administración sin sesión y con rol cliente</x:v>
-      </x:c>
-      <x:c r="G41" s="44" t="str">
-        <x:v>Visitante va a login; cliente vuelve a Inicio</x:v>
-      </x:c>
-      <x:c r="H41" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I41" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J41" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K41" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L41" s="44" t="str">
-        <x:v>Duración: 12 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A42" s="44" t="str">
-        <x:v>PU-041</x:v>
-      </x:c>
-      <x:c r="B42" s="44" t="str">
-        <x:v>Checkout</x:v>
-      </x:c>
-      <x:c r="C42" s="44" t="str">
-        <x:v>Estado de campos</x:v>
-      </x:c>
-      <x:c r="D42" s="44" t="str">
-        <x:v>Normal</x:v>
-      </x:c>
-      <x:c r="E42" s="44" t="str">
-        <x:v>Checkout precarga sesión y mantiene estado de campos</x:v>
-      </x:c>
-      <x:c r="F42" s="44" t="str">
-        <x:v>Cliente autenticado y dirección editada</x:v>
-      </x:c>
-      <x:c r="G42" s="44" t="str">
-        <x:v>Nombre precargado y dirección nueva reflejada en el input</x:v>
-      </x:c>
-      <x:c r="H42" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I42" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J42" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K42" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L42" s="44" t="str">
-        <x:v>Duración: 27 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A43" s="44" t="str">
-        <x:v>PU-042</x:v>
-      </x:c>
-      <x:c r="B43" s="44" t="str">
-        <x:v>Checkout</x:v>
-      </x:c>
-      <x:c r="C43" s="44" t="str">
-        <x:v>Confirmar compra</x:v>
-      </x:c>
-      <x:c r="D43" s="44" t="str">
-        <x:v>Normal</x:v>
-      </x:c>
-      <x:c r="E43" s="44" t="str">
-        <x:v>Checkout aprobado confirma y vacía el carrito</x:v>
-      </x:c>
-      <x:c r="F43" s="44" t="str">
-        <x:v>Datos precargados y confirmación de compra</x:v>
-      </x:c>
-      <x:c r="G43" s="44" t="str">
-        <x:v>Una orden, vista de confirmación y carrito vacío</x:v>
-      </x:c>
-      <x:c r="H43" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I43" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J43" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K43" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L43" s="44" t="str">
-        <x:v>Duración: 27 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A44" s="44" t="str">
-        <x:v>PU-043</x:v>
-      </x:c>
-      <x:c r="B44" s="44" t="str">
-        <x:v>Checkout</x:v>
-      </x:c>
-      <x:c r="C44" s="44" t="str">
-        <x:v>Rechazar pago</x:v>
-      </x:c>
-      <x:c r="D44" s="44" t="str">
-        <x:v>Error</x:v>
-      </x:c>
-      <x:c r="E44" s="44" t="str">
-        <x:v>Checkout rechazado conserva el carrito</x:v>
-      </x:c>
-      <x:c r="F44" s="44" t="str">
-        <x:v>Elegir pago rechazado</x:v>
-      </x:c>
-      <x:c r="G44" s="44" t="str">
-        <x:v>Vista de rechazo; carrito intacto y sin pedido</x:v>
-      </x:c>
-      <x:c r="H44" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I44" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J44" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K44" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L44" s="44" t="str">
-        <x:v>Duración: 11 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A45" s="44" t="str">
-        <x:v>PU-044</x:v>
-      </x:c>
-      <x:c r="B45" s="44" t="str">
-        <x:v>PerfilUsuario</x:v>
-      </x:c>
-      <x:c r="C45" s="44" t="str">
-        <x:v>Filtro de historial</x:v>
-      </x:c>
-      <x:c r="D45" s="44" t="str">
-        <x:v>Normal</x:v>
-      </x:c>
-      <x:c r="E45" s="44" t="str">
-        <x:v>Perfil filtra el historial por la cuenta activa</x:v>
-      </x:c>
-      <x:c r="F45" s="44" t="str">
-        <x:v>Dos pedidos con correos diferentes y usuario Ana</x:v>
-      </x:c>
-      <x:c r="G45" s="44" t="str">
-        <x:v>Muestra solamente el pedido de Ana</x:v>
-      </x:c>
-      <x:c r="H45" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I45" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J45" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K45" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L45" s="44" t="str">
-        <x:v>Duración: 23 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A46" s="44" t="str">
-        <x:v>PU-045</x:v>
-      </x:c>
-      <x:c r="B46" s="44" t="str">
-        <x:v>Compra</x:v>
-      </x:c>
-      <x:c r="C46" s="44" t="str">
-        <x:v>Pedido inexistente</x:v>
-      </x:c>
-      <x:c r="D46" s="44" t="str">
-        <x:v>Error</x:v>
-      </x:c>
-      <x:c r="E46" s="44" t="str">
-        <x:v>Resumen de compra maneja pedidos inexistentes</x:v>
-      </x:c>
-      <x:c r="F46" s="44" t="str">
-        <x:v>URL /compra/no-existe</x:v>
-      </x:c>
-      <x:c r="G46" s="44" t="str">
-        <x:v>Mensaje de pedido no disponible</x:v>
-      </x:c>
-      <x:c r="H46" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I46" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J46" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K46" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L46" s="44" t="str">
-        <x:v>Duración: 3 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A47" s="44" t="str">
-        <x:v>PU-046</x:v>
-      </x:c>
-      <x:c r="B47" s="44" t="str">
-        <x:v>Ofertas</x:v>
-      </x:c>
-      <x:c r="C47" s="44" t="str">
-        <x:v>Filtro de descuentos</x:v>
-      </x:c>
-      <x:c r="D47" s="44" t="str">
-        <x:v>Normal</x:v>
-      </x:c>
-      <x:c r="E47" s="44" t="str">
-        <x:v>Ofertas excluye productos sin descuento</x:v>
-      </x:c>
-      <x:c r="F47" s="44" t="str">
-        <x:v>Dos productos; uno con 20% y otro con descuento cero</x:v>
-      </x:c>
-      <x:c r="G47" s="44" t="str">
-        <x:v>Una sola tarjeta con precio 8000</x:v>
-      </x:c>
-      <x:c r="H47" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I47" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J47" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K47" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L47" s="44" t="str">
-        <x:v>Duración: 11 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48" ht="78.75" hidden="0" customHeight="1">
-      <x:c r="A48" s="44" t="str">
-        <x:v>PU-047</x:v>
-      </x:c>
-      <x:c r="B48" s="44" t="str">
-        <x:v>Categorias</x:v>
-      </x:c>
-      <x:c r="C48" s="44" t="str">
-        <x:v>Renderizado y enlaces</x:v>
-      </x:c>
-      <x:c r="D48" s="44" t="str">
-        <x:v>Normal</x:v>
-      </x:c>
-      <x:c r="E48" s="44" t="str">
-        <x:v>Categorías renderiza el conjunto disponible</x:v>
-      </x:c>
-      <x:c r="F48" s="44" t="str">
-        <x:v>Cuatro categorías y catálogo inicial</x:v>
-      </x:c>
-      <x:c r="G48" s="44" t="str">
-        <x:v>Cuatro tarjetas con enlaces y tres productos por categoría</x:v>
-      </x:c>
-      <x:c r="H48" s="44" t="str">
-        <x:v>Todas las aserciones del caso se aprobaron</x:v>
-      </x:c>
-      <x:c r="I48" s="44" t="str">
-        <x:v>Pasó</x:v>
-      </x:c>
-      <x:c r="J48" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
-      </x:c>
-      <x:c r="K48" s="46" t="d">
-        <x:v>2026-10-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L48" s="44" t="str">
-        <x:v>Duración: 3 ms. Chrome Headless 155.0.0.0 (Windows 10)</x:v>
-      </x:c>
+    <x:row r="12" ht="15" hidden="0">
+      <x:c r="A12" s="8"/>
+      <x:c r="B12" s="8"/>
+      <x:c r="C12" s="8"/>
+      <x:c r="D12" s="8"/>
+      <x:c r="E12" s="8"/>
+      <x:c r="F12" s="8"/>
+      <x:c r="G12" s="8"/>
+      <x:c r="H12" s="8"/>
+      <x:c r="I12" s="8"/>
+      <x:c r="J12" s="8"/>
+      <x:c r="K12" s="9"/>
+      <x:c r="L12" s="8"/>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0">
+      <x:c r="A13" s="8"/>
+      <x:c r="B13" s="8"/>
+      <x:c r="C13" s="8"/>
+      <x:c r="D13" s="8"/>
+      <x:c r="E13" s="8"/>
+      <x:c r="F13" s="8"/>
+      <x:c r="G13" s="8"/>
+      <x:c r="H13" s="8"/>
+      <x:c r="I13" s="8"/>
+      <x:c r="J13" s="8"/>
+      <x:c r="K13" s="9"/>
+      <x:c r="L13" s="8"/>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0">
+      <x:c r="A14" s="8"/>
+      <x:c r="B14" s="8"/>
+      <x:c r="C14" s="8"/>
+      <x:c r="D14" s="8"/>
+      <x:c r="E14" s="8"/>
+      <x:c r="F14" s="8"/>
+      <x:c r="G14" s="8"/>
+      <x:c r="H14" s="8"/>
+      <x:c r="I14" s="8"/>
+      <x:c r="J14" s="8"/>
+      <x:c r="K14" s="9"/>
+      <x:c r="L14" s="8"/>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0">
+      <x:c r="A15" s="8"/>
+      <x:c r="B15" s="8"/>
+      <x:c r="C15" s="8"/>
+      <x:c r="D15" s="8"/>
+      <x:c r="E15" s="8"/>
+      <x:c r="F15" s="8"/>
+      <x:c r="G15" s="8"/>
+      <x:c r="H15" s="8"/>
+      <x:c r="I15" s="8"/>
+      <x:c r="J15" s="8"/>
+      <x:c r="K15" s="9"/>
+      <x:c r="L15" s="8"/>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0">
+      <x:c r="A16" s="8"/>
+      <x:c r="B16" s="8"/>
+      <x:c r="C16" s="8"/>
+      <x:c r="D16" s="8"/>
+      <x:c r="E16" s="8"/>
+      <x:c r="F16" s="8"/>
+      <x:c r="G16" s="8"/>
+      <x:c r="H16" s="8"/>
+      <x:c r="I16" s="8"/>
+      <x:c r="J16" s="8"/>
+      <x:c r="K16" s="9"/>
+      <x:c r="L16" s="8"/>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0">
+      <x:c r="A17" s="8"/>
+      <x:c r="B17" s="8"/>
+      <x:c r="C17" s="8"/>
+      <x:c r="D17" s="8"/>
+      <x:c r="E17" s="8"/>
+      <x:c r="F17" s="8"/>
+      <x:c r="G17" s="8"/>
+      <x:c r="H17" s="8"/>
+      <x:c r="I17" s="8"/>
+      <x:c r="J17" s="8"/>
+      <x:c r="K17" s="9"/>
+      <x:c r="L17" s="8"/>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0">
+      <x:c r="A18" s="8"/>
+      <x:c r="B18" s="8"/>
+      <x:c r="C18" s="8"/>
+      <x:c r="D18" s="8"/>
+      <x:c r="E18" s="8"/>
+      <x:c r="F18" s="8"/>
+      <x:c r="G18" s="8"/>
+      <x:c r="H18" s="8"/>
+      <x:c r="I18" s="8"/>
+      <x:c r="J18" s="8"/>
+      <x:c r="K18" s="9"/>
+      <x:c r="L18" s="8"/>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0">
+      <x:c r="A19" s="8"/>
+      <x:c r="B19" s="8"/>
+      <x:c r="C19" s="8"/>
+      <x:c r="D19" s="8"/>
+      <x:c r="E19" s="8"/>
+      <x:c r="F19" s="8"/>
+      <x:c r="G19" s="8"/>
+      <x:c r="H19" s="8"/>
+      <x:c r="I19" s="8"/>
+      <x:c r="J19" s="8"/>
+      <x:c r="K19" s="9"/>
+      <x:c r="L19" s="8"/>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0">
+      <x:c r="A20" s="8"/>
+      <x:c r="B20" s="8"/>
+      <x:c r="C20" s="8"/>
+      <x:c r="D20" s="8"/>
+      <x:c r="E20" s="8"/>
+      <x:c r="F20" s="8"/>
+      <x:c r="G20" s="8"/>
+      <x:c r="H20" s="8"/>
+      <x:c r="I20" s="8"/>
+      <x:c r="J20" s="8"/>
+      <x:c r="K20" s="9"/>
+      <x:c r="L20" s="8"/>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0">
+      <x:c r="A21" s="8"/>
+      <x:c r="B21" s="8"/>
+      <x:c r="C21" s="8"/>
+      <x:c r="D21" s="8"/>
+      <x:c r="E21" s="8"/>
+      <x:c r="F21" s="8"/>
+      <x:c r="G21" s="8"/>
+      <x:c r="H21" s="8"/>
+      <x:c r="I21" s="8"/>
+      <x:c r="J21" s="8"/>
+      <x:c r="K21" s="9"/>
+      <x:c r="L21" s="8"/>
+    </x:row>
+    <x:row r="22" ht="15" hidden="0">
+      <x:c r="A22" s="8"/>
+      <x:c r="B22" s="8"/>
+      <x:c r="C22" s="8"/>
+      <x:c r="D22" s="8"/>
+      <x:c r="E22" s="8"/>
+      <x:c r="F22" s="8"/>
+      <x:c r="G22" s="8"/>
+      <x:c r="H22" s="8"/>
+      <x:c r="I22" s="8"/>
+      <x:c r="J22" s="8"/>
+      <x:c r="K22" s="9"/>
+      <x:c r="L22" s="8"/>
+    </x:row>
+    <x:row r="23" ht="15" hidden="0">
+      <x:c r="A23" s="8"/>
+      <x:c r="B23" s="8"/>
+      <x:c r="C23" s="8"/>
+      <x:c r="D23" s="8"/>
+      <x:c r="E23" s="8"/>
+      <x:c r="F23" s="8"/>
+      <x:c r="G23" s="8"/>
+      <x:c r="H23" s="8"/>
+      <x:c r="I23" s="8"/>
+      <x:c r="J23" s="8"/>
+      <x:c r="K23" s="9"/>
+      <x:c r="L23" s="8"/>
+    </x:row>
+    <x:row r="24" ht="15" hidden="0">
+      <x:c r="A24" s="8"/>
+      <x:c r="B24" s="8"/>
+      <x:c r="C24" s="8"/>
+      <x:c r="D24" s="8"/>
+      <x:c r="E24" s="8"/>
+      <x:c r="F24" s="8"/>
+      <x:c r="G24" s="8"/>
+      <x:c r="H24" s="8"/>
+      <x:c r="I24" s="8"/>
+      <x:c r="J24" s="8"/>
+      <x:c r="K24" s="9"/>
+      <x:c r="L24" s="8"/>
+    </x:row>
+    <x:row r="25" ht="15" hidden="0">
+      <x:c r="A25" s="8"/>
+      <x:c r="B25" s="8"/>
+      <x:c r="C25" s="8"/>
+      <x:c r="D25" s="8"/>
+      <x:c r="E25" s="8"/>
+      <x:c r="F25" s="8"/>
+      <x:c r="G25" s="8"/>
+      <x:c r="H25" s="8"/>
+      <x:c r="I25" s="8"/>
+      <x:c r="J25" s="8"/>
+      <x:c r="K25" s="9"/>
+      <x:c r="L25" s="8"/>
+    </x:row>
+    <x:row r="26" ht="15" hidden="0">
+      <x:c r="A26" s="8"/>
+      <x:c r="B26" s="8"/>
+      <x:c r="C26" s="8"/>
+      <x:c r="D26" s="8"/>
+      <x:c r="E26" s="8"/>
+      <x:c r="F26" s="8"/>
+      <x:c r="G26" s="8"/>
+      <x:c r="H26" s="8"/>
+      <x:c r="I26" s="8"/>
+      <x:c r="J26" s="8"/>
+      <x:c r="K26" s="9"/>
+      <x:c r="L26" s="8"/>
+    </x:row>
+    <x:row r="27" ht="15" hidden="0">
+      <x:c r="A27" s="8"/>
+      <x:c r="B27" s="8"/>
+      <x:c r="C27" s="8"/>
+      <x:c r="D27" s="8"/>
+      <x:c r="E27" s="8"/>
+      <x:c r="F27" s="8"/>
+      <x:c r="G27" s="8"/>
+      <x:c r="H27" s="8"/>
+      <x:c r="I27" s="8"/>
+      <x:c r="J27" s="8"/>
+      <x:c r="K27" s="9"/>
+      <x:c r="L27" s="8"/>
+    </x:row>
+    <x:row r="28" ht="15" hidden="0">
+      <x:c r="A28" s="8"/>
+      <x:c r="B28" s="8"/>
+      <x:c r="C28" s="8"/>
+      <x:c r="D28" s="8"/>
+      <x:c r="E28" s="8"/>
+      <x:c r="F28" s="8"/>
+      <x:c r="G28" s="8"/>
+      <x:c r="H28" s="8"/>
+      <x:c r="I28" s="8"/>
+      <x:c r="J28" s="8"/>
+      <x:c r="K28" s="9"/>
+      <x:c r="L28" s="8"/>
+    </x:row>
+    <x:row r="29" ht="15" hidden="0">
+      <x:c r="A29" s="8"/>
+      <x:c r="B29" s="8"/>
+      <x:c r="C29" s="8"/>
+      <x:c r="D29" s="8"/>
+      <x:c r="E29" s="8"/>
+      <x:c r="F29" s="8"/>
+      <x:c r="G29" s="8"/>
+      <x:c r="H29" s="8"/>
+      <x:c r="I29" s="8"/>
+      <x:c r="J29" s="8"/>
+      <x:c r="K29" s="9"/>
+      <x:c r="L29" s="8"/>
+    </x:row>
+    <x:row r="30" ht="15" hidden="0">
+      <x:c r="A30" s="8"/>
+      <x:c r="B30" s="8"/>
+      <x:c r="C30" s="8"/>
+      <x:c r="D30" s="8"/>
+      <x:c r="E30" s="8"/>
+      <x:c r="F30" s="8"/>
+      <x:c r="G30" s="8"/>
+      <x:c r="H30" s="8"/>
+      <x:c r="I30" s="8"/>
+      <x:c r="J30" s="8"/>
+      <x:c r="K30" s="9"/>
+      <x:c r="L30" s="8"/>
+    </x:row>
+    <x:row r="31" ht="15" hidden="0">
+      <x:c r="A31" s="8"/>
+      <x:c r="B31" s="8"/>
+      <x:c r="C31" s="8"/>
+      <x:c r="D31" s="8"/>
+      <x:c r="E31" s="8"/>
+      <x:c r="F31" s="8"/>
+      <x:c r="G31" s="8"/>
+      <x:c r="H31" s="8"/>
+      <x:c r="I31" s="8"/>
+      <x:c r="J31" s="8"/>
+      <x:c r="K31" s="9"/>
+      <x:c r="L31" s="8"/>
+    </x:row>
+    <x:row r="32" ht="15" hidden="0">
+      <x:c r="A32" s="8"/>
+      <x:c r="B32" s="8"/>
+      <x:c r="C32" s="8"/>
+      <x:c r="D32" s="8"/>
+      <x:c r="E32" s="8"/>
+      <x:c r="F32" s="8"/>
+      <x:c r="G32" s="8"/>
+      <x:c r="H32" s="8"/>
+      <x:c r="I32" s="8"/>
+      <x:c r="J32" s="8"/>
+      <x:c r="K32" s="9"/>
+      <x:c r="L32" s="8"/>
+    </x:row>
+    <x:row r="33" ht="15" hidden="0">
+      <x:c r="A33" s="8"/>
+      <x:c r="B33" s="8"/>
+      <x:c r="C33" s="8"/>
+      <x:c r="D33" s="8"/>
+      <x:c r="E33" s="8"/>
+      <x:c r="F33" s="8"/>
+      <x:c r="G33" s="8"/>
+      <x:c r="H33" s="8"/>
+      <x:c r="I33" s="8"/>
+      <x:c r="J33" s="8"/>
+      <x:c r="K33" s="9"/>
+      <x:c r="L33" s="8"/>
+    </x:row>
+    <x:row r="34" ht="15" hidden="0">
+      <x:c r="A34" s="8"/>
+      <x:c r="B34" s="8"/>
+      <x:c r="C34" s="8"/>
+      <x:c r="D34" s="8"/>
+      <x:c r="E34" s="8"/>
+      <x:c r="F34" s="8"/>
+      <x:c r="G34" s="8"/>
+      <x:c r="H34" s="8"/>
+      <x:c r="I34" s="8"/>
+      <x:c r="J34" s="8"/>
+      <x:c r="K34" s="9"/>
+      <x:c r="L34" s="8"/>
+    </x:row>
+    <x:row r="35" ht="15" hidden="0">
+      <x:c r="A35" s="8"/>
+      <x:c r="B35" s="8"/>
+      <x:c r="C35" s="8"/>
+      <x:c r="D35" s="8"/>
+      <x:c r="E35" s="8"/>
+      <x:c r="F35" s="8"/>
+      <x:c r="G35" s="8"/>
+      <x:c r="H35" s="8"/>
+      <x:c r="I35" s="8"/>
+      <x:c r="J35" s="8"/>
+      <x:c r="K35" s="9"/>
+      <x:c r="L35" s="8"/>
+    </x:row>
+    <x:row r="36" ht="15" hidden="0">
+      <x:c r="A36" s="8"/>
+      <x:c r="B36" s="8"/>
+      <x:c r="C36" s="8"/>
+      <x:c r="D36" s="8"/>
+      <x:c r="E36" s="8"/>
+      <x:c r="F36" s="8"/>
+      <x:c r="G36" s="8"/>
+      <x:c r="H36" s="8"/>
+      <x:c r="I36" s="8"/>
+      <x:c r="J36" s="8"/>
+      <x:c r="K36" s="9"/>
+      <x:c r="L36" s="8"/>
+    </x:row>
+    <x:row r="37" ht="15" hidden="0">
+      <x:c r="A37" s="8"/>
+      <x:c r="B37" s="8"/>
+      <x:c r="C37" s="8"/>
+      <x:c r="D37" s="8"/>
+      <x:c r="E37" s="8"/>
+      <x:c r="F37" s="8"/>
+      <x:c r="G37" s="8"/>
+      <x:c r="H37" s="8"/>
+      <x:c r="I37" s="8"/>
+      <x:c r="J37" s="8"/>
+      <x:c r="K37" s="9"/>
+      <x:c r="L37" s="8"/>
+    </x:row>
+    <x:row r="38" ht="15" hidden="0">
+      <x:c r="A38" s="8"/>
+      <x:c r="B38" s="8"/>
+      <x:c r="C38" s="8"/>
+      <x:c r="D38" s="8"/>
+      <x:c r="E38" s="8"/>
+      <x:c r="F38" s="8"/>
+      <x:c r="G38" s="8"/>
+      <x:c r="H38" s="8"/>
+      <x:c r="I38" s="8"/>
+      <x:c r="J38" s="8"/>
+      <x:c r="K38" s="9"/>
+      <x:c r="L38" s="8"/>
+    </x:row>
+    <x:row r="39" ht="15" hidden="0">
+      <x:c r="A39" s="8"/>
+      <x:c r="B39" s="8"/>
+      <x:c r="C39" s="8"/>
+      <x:c r="D39" s="8"/>
+      <x:c r="E39" s="8"/>
+      <x:c r="F39" s="8"/>
+      <x:c r="G39" s="8"/>
+      <x:c r="H39" s="8"/>
+      <x:c r="I39" s="8"/>
+      <x:c r="J39" s="8"/>
+      <x:c r="K39" s="9"/>
+      <x:c r="L39" s="8"/>
+    </x:row>
+    <x:row r="40" ht="15" hidden="0">
+      <x:c r="A40" s="8"/>
+      <x:c r="B40" s="8"/>
+      <x:c r="C40" s="8"/>
+      <x:c r="D40" s="8"/>
+      <x:c r="E40" s="8"/>
+      <x:c r="F40" s="8"/>
+      <x:c r="G40" s="8"/>
+      <x:c r="H40" s="8"/>
+      <x:c r="I40" s="8"/>
+      <x:c r="J40" s="8"/>
+      <x:c r="K40" s="9"/>
+      <x:c r="L40" s="8"/>
+    </x:row>
+    <x:row r="41" ht="15" hidden="0">
+      <x:c r="A41" s="8"/>
+      <x:c r="B41" s="8"/>
+      <x:c r="C41" s="8"/>
+      <x:c r="D41" s="8"/>
+      <x:c r="E41" s="8"/>
+      <x:c r="F41" s="8"/>
+      <x:c r="G41" s="8"/>
+      <x:c r="H41" s="8"/>
+      <x:c r="I41" s="8"/>
+      <x:c r="J41" s="8"/>
+      <x:c r="K41" s="9"/>
+      <x:c r="L41" s="8"/>
+    </x:row>
+    <x:row r="42" ht="15" hidden="0">
+      <x:c r="A42" s="8"/>
+      <x:c r="B42" s="8"/>
+      <x:c r="C42" s="8"/>
+      <x:c r="D42" s="8"/>
+      <x:c r="E42" s="8"/>
+      <x:c r="F42" s="8"/>
+      <x:c r="G42" s="8"/>
+      <x:c r="H42" s="8"/>
+      <x:c r="I42" s="8"/>
+      <x:c r="J42" s="8"/>
+      <x:c r="K42" s="9"/>
+      <x:c r="L42" s="8"/>
+    </x:row>
+    <x:row r="43" ht="15" hidden="0">
+      <x:c r="A43" s="8"/>
+      <x:c r="B43" s="8"/>
+      <x:c r="C43" s="8"/>
+      <x:c r="D43" s="8"/>
+      <x:c r="E43" s="8"/>
+      <x:c r="F43" s="8"/>
+      <x:c r="G43" s="8"/>
+      <x:c r="H43" s="8"/>
+      <x:c r="I43" s="8"/>
+      <x:c r="J43" s="8"/>
+      <x:c r="K43" s="9"/>
+      <x:c r="L43" s="8"/>
+    </x:row>
+    <x:row r="44" ht="15" hidden="0">
+      <x:c r="A44" s="8"/>
+      <x:c r="B44" s="8"/>
+      <x:c r="C44" s="8"/>
+      <x:c r="D44" s="8"/>
+      <x:c r="E44" s="8"/>
+      <x:c r="F44" s="8"/>
+      <x:c r="G44" s="8"/>
+      <x:c r="H44" s="8"/>
+      <x:c r="I44" s="8"/>
+      <x:c r="J44" s="8"/>
+      <x:c r="K44" s="9"/>
+      <x:c r="L44" s="8"/>
+    </x:row>
+    <x:row r="45" ht="15" hidden="0">
+      <x:c r="A45" s="8"/>
+      <x:c r="B45" s="8"/>
+      <x:c r="C45" s="8"/>
+      <x:c r="D45" s="8"/>
+      <x:c r="E45" s="8"/>
+      <x:c r="F45" s="8"/>
+      <x:c r="G45" s="8"/>
+      <x:c r="H45" s="8"/>
+      <x:c r="I45" s="8"/>
+      <x:c r="J45" s="8"/>
+      <x:c r="K45" s="9"/>
+      <x:c r="L45" s="8"/>
+    </x:row>
+    <x:row r="46" ht="15" hidden="0">
+      <x:c r="A46" s="8"/>
+      <x:c r="B46" s="8"/>
+      <x:c r="C46" s="8"/>
+      <x:c r="D46" s="8"/>
+      <x:c r="E46" s="8"/>
+      <x:c r="F46" s="8"/>
+      <x:c r="G46" s="8"/>
+      <x:c r="H46" s="8"/>
+      <x:c r="I46" s="8"/>
+      <x:c r="J46" s="8"/>
+      <x:c r="K46" s="9"/>
+      <x:c r="L46" s="8"/>
+    </x:row>
+    <x:row r="47" ht="15" hidden="0">
+      <x:c r="A47" s="8"/>
+      <x:c r="B47" s="8"/>
+      <x:c r="C47" s="8"/>
+      <x:c r="D47" s="8"/>
+      <x:c r="E47" s="8"/>
+      <x:c r="F47" s="8"/>
+      <x:c r="G47" s="8"/>
+      <x:c r="H47" s="8"/>
+      <x:c r="I47" s="8"/>
+      <x:c r="J47" s="8"/>
+      <x:c r="K47" s="9"/>
+      <x:c r="L47" s="8"/>
+    </x:row>
+    <x:row r="48" ht="15" hidden="0">
+      <x:c r="A48" s="8"/>
+      <x:c r="B48" s="8"/>
+      <x:c r="C48" s="8"/>
+      <x:c r="D48" s="8"/>
+      <x:c r="E48" s="8"/>
+      <x:c r="F48" s="8"/>
+      <x:c r="G48" s="8"/>
+      <x:c r="H48" s="8"/>
+      <x:c r="I48" s="8"/>
+      <x:c r="J48" s="8"/>
+      <x:c r="K48" s="9"/>
+      <x:c r="L48" s="8"/>
     </x:row>
     <x:row r="49" ht="15" hidden="0">
       <x:c r="A49" s="8"/>
@@ -5102,25 +4214,25 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:dataValidations count="4">
-    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="I49:I201">
+    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="I12:I201">
       <x:formula1>"Pasó,Falló,Pendiente,Omitido"</x:formula1>
       <x:formula2>0</x:formula2>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D49:D201">
+    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D12:D201">
       <x:formula1>"Normal,Borde,Error"</x:formula1>
       <x:formula2>0</x:formula2>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="I2:I48">
+    <x:dataValidation type="list" errorStyle="stop" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="I2:I11">
       <x:formula1>"Pasó,Falló,Pendiente,Omitido"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D2:D48">
+    <x:dataValidation type="list" errorStyle="stop" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D2:D11">
       <x:formula1>"Normal,Borde,Error"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c44a4555cab448c"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c063b15289a44c0"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec0fde2a3ade49d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6845a785c8164b97"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5145,8 +4257,8 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="B3" s="47" t="n">
-        <x:f aca="0">COUNTA('Casos de Prueba'!A2:A48)</x:f>
-        <x:v>47</x:v>
+        <x:f aca="0">COUNTA('Casos de Prueba'!A2:A11)</x:f>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="21.75" hidden="0" customHeight="1">
@@ -5154,8 +4266,8 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="B4" s="47" t="n">
-        <x:f aca="0">COUNTIFS('Casos de Prueba'!I2:I48,A4)</x:f>
-        <x:v>47</x:v>
+        <x:f aca="0">COUNTIFS('Casos de Prueba'!I2:I11,A4)</x:f>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="21.75" hidden="0" customHeight="1">
@@ -5163,7 +4275,7 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="B5" s="47" t="n">
-        <x:f aca="0">COUNTIFS('Casos de Prueba'!I2:I48,A5)</x:f>
+        <x:f aca="0">COUNTIFS('Casos de Prueba'!I2:I11,A5)</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -5172,7 +4284,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="B6" s="47" t="n">
-        <x:f aca="0">COUNTIFS('Casos de Prueba'!I2:I48,A6)</x:f>
+        <x:f aca="0">COUNTIFS('Casos de Prueba'!I2:I11,A6)</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -5181,7 +4293,7 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="B7" s="47" t="n">
-        <x:f aca="0">COUNTIFS('Casos de Prueba'!I2:I48,A7)</x:f>
+        <x:f aca="0">COUNTIFS('Casos de Prueba'!I2:I11,A7)</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -5237,11 +4349,11 @@
       </x:c>
       <x:c r="B15" s="11" t="n">
         <x:f aca="0">COUNTIF('Casos de Prueba'!D2:D201,A15)</x:f>
-        <x:v>24</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C15" s="11" t="n">
         <x:f aca="0">COUNTIFS('Casos de Prueba'!D2:D201,A15,'Casos de Prueba'!I2:I201,"Pasó")</x:f>
-        <x:v>24</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D15" s="11" t="n">
         <x:f aca="0">COUNTIFS('Casos de Prueba'!D2:D201,A15,'Casos de Prueba'!I2:I201,"Falló")</x:f>
@@ -5254,11 +4366,11 @@
       </x:c>
       <x:c r="B16" s="11" t="n">
         <x:f aca="0">COUNTIF('Casos de Prueba'!D2:D201,A16)</x:f>
-        <x:v>7</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C16" s="11" t="n">
         <x:f aca="0">COUNTIFS('Casos de Prueba'!D2:D201,A16,'Casos de Prueba'!I2:I201,"Pasó")</x:f>
-        <x:v>7</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D16" s="11" t="n">
         <x:f aca="0">COUNTIFS('Casos de Prueba'!D2:D201,A16,'Casos de Prueba'!I2:I201,"Falló")</x:f>
@@ -5271,11 +4383,11 @@
       </x:c>
       <x:c r="B17" s="11" t="n">
         <x:f aca="0">COUNTIF('Casos de Prueba'!D2:D201,A17)</x:f>
-        <x:v>16</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C17" s="11" t="n">
         <x:f aca="0">COUNTIFS('Casos de Prueba'!D2:D201,A17,'Casos de Prueba'!I2:I201,"Pasó")</x:f>
-        <x:v>16</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D17" s="11" t="n">
         <x:f aca="0">COUNTIFS('Casos de Prueba'!D2:D201,A17,'Casos de Prueba'!I2:I201,"Falló")</x:f>

</xml_diff>

<commit_message>
Corrige los nombres completos de los responsables
Actualiza la guía, la ERS y la planilla de pruebas con Diego Roble, Victoria Arias y Vicente Perez como equipo responsable.
</commit_message>
<xml_diff>
--- a/docs/Registro_Pruebas_Unitarias.xlsx
+++ b/docs/Registro_Pruebas_Unitarias.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" r:id="Rc7da2d5bc8f64cb4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos de Prueba" sheetId="2" r:id="R34549a4d57974547"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="3" r:id="Ra0c253c08ff14a84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" r:id="R81fea57214454e93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos de Prueba" sheetId="2" r:id="Rfd512bb5a2704ea3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="3" r:id="R26984d214815451c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -971,7 +971,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B5" s="33" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
+        <x:v>Diego Roble, Victoria Arias y Vicente Perez</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0">
@@ -1093,7 +1093,7 @@
         <x:v>Responsables:</x:v>
       </x:c>
       <x:c r="B25" s="35" t="str">
-        <x:v>Equipo conjunto: Vicente, Victoria y Diego. Sin asignación individual de casos.</x:v>
+        <x:v>Equipo conjunto: Diego Roble, Victoria Arias y Vicente Perez. Sin asignación individual de casos.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1187,7 +1187,7 @@
         <x:v>Pasó</x:v>
       </x:c>
       <x:c r="J2" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
+        <x:v>Diego Roble, Victoria Arias y Vicente Perez</x:v>
       </x:c>
       <x:c r="K2" s="46" t="d">
         <x:v>2026-10-14T00:00:00.000Z</x:v>
@@ -1225,7 +1225,7 @@
         <x:v>Pasó</x:v>
       </x:c>
       <x:c r="J3" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
+        <x:v>Diego Roble, Victoria Arias y Vicente Perez</x:v>
       </x:c>
       <x:c r="K3" s="46" t="d">
         <x:v>2026-10-14T00:00:00.000Z</x:v>
@@ -1263,7 +1263,7 @@
         <x:v>Pasó</x:v>
       </x:c>
       <x:c r="J4" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
+        <x:v>Diego Roble, Victoria Arias y Vicente Perez</x:v>
       </x:c>
       <x:c r="K4" s="46" t="d">
         <x:v>2026-10-14T00:00:00.000Z</x:v>
@@ -1301,7 +1301,7 @@
         <x:v>Pasó</x:v>
       </x:c>
       <x:c r="J5" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
+        <x:v>Diego Roble, Victoria Arias y Vicente Perez</x:v>
       </x:c>
       <x:c r="K5" s="46" t="d">
         <x:v>2026-10-14T00:00:00.000Z</x:v>
@@ -1339,7 +1339,7 @@
         <x:v>Pasó</x:v>
       </x:c>
       <x:c r="J6" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
+        <x:v>Diego Roble, Victoria Arias y Vicente Perez</x:v>
       </x:c>
       <x:c r="K6" s="46" t="d">
         <x:v>2026-10-14T00:00:00.000Z</x:v>
@@ -1377,7 +1377,7 @@
         <x:v>Pasó</x:v>
       </x:c>
       <x:c r="J7" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
+        <x:v>Diego Roble, Victoria Arias y Vicente Perez</x:v>
       </x:c>
       <x:c r="K7" s="46" t="d">
         <x:v>2026-10-14T00:00:00.000Z</x:v>
@@ -1415,7 +1415,7 @@
         <x:v>Pasó</x:v>
       </x:c>
       <x:c r="J8" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
+        <x:v>Diego Roble, Victoria Arias y Vicente Perez</x:v>
       </x:c>
       <x:c r="K8" s="46" t="d">
         <x:v>2026-10-14T00:00:00.000Z</x:v>
@@ -1453,7 +1453,7 @@
         <x:v>Pasó</x:v>
       </x:c>
       <x:c r="J9" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
+        <x:v>Diego Roble, Victoria Arias y Vicente Perez</x:v>
       </x:c>
       <x:c r="K9" s="46" t="d">
         <x:v>2026-10-14T00:00:00.000Z</x:v>
@@ -1491,7 +1491,7 @@
         <x:v>Pasó</x:v>
       </x:c>
       <x:c r="J10" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
+        <x:v>Diego Roble, Victoria Arias y Vicente Perez</x:v>
       </x:c>
       <x:c r="K10" s="46" t="d">
         <x:v>2026-10-14T00:00:00.000Z</x:v>
@@ -1529,7 +1529,7 @@
         <x:v>Pasó</x:v>
       </x:c>
       <x:c r="J11" s="44" t="str">
-        <x:v>Vicente, Victoria y Diego</x:v>
+        <x:v>Diego Roble, Victoria Arias y Vicente Perez</x:v>
       </x:c>
       <x:c r="K11" s="46" t="d">
         <x:v>2026-10-14T00:00:00.000Z</x:v>
@@ -4230,9 +4230,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c063b15289a44c0"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32c16438675345e4"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6845a785c8164b97"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f9d11d938094234"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>